<commit_message>
Escala o módulo de proteção solar e verão (universo vai a 379 termos)
Mantém o universo de esporte por jornada e adiciona um hub próprio de proteção
solar e verão, amplo e não colado a esporte: fundamentos (o que é FPS/UPF/UV50),
roupa UV (proposta de valor da marca), protetor solar (adjacente), pele e saúde
(prevenção, autoridade), proteção infantil, dicas da estação e look de verão.
371 termos novos em 4 lotes de 100 para medir no Semrush.
</commit_message>
<xml_diff>
--- a/data/2026-08-12-universo-esporte-jornada.xlsx
+++ b/data/2026-08-12-universo-esporte-jornada.xlsx
@@ -11,7 +11,8 @@
     <sheet name="Semrush lote 1" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Semrush lote 2" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Semrush lote 3" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="resumo" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Semrush lote 4" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="resumo" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -429,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E290"/>
+  <dimension ref="A1:E380"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -8264,6 +8265,2436 @@
         </is>
       </c>
       <c r="E290" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>o que é fps</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>Fundamento</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>o que é fpu</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>Fundamento</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>o que é upf</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>Fundamento</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>o que significa uv50</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>Fundamento</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>diferença entre uva e uvb</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Fundamento</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>o que é índice uv</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Fundamento</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>o que é radiação ultravioleta</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Fundamento</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>o que é fotoproteção</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>Fundamento</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>fps qual o ideal</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Fundamento</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>fps 30 ou 50</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Fundamento</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>o que é fator de proteção uv na roupa</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Fundamento</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>roupa com proteção solar</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Comercial</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>roupa com proteção uv</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>Comercial</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>roupa com fps</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>Comercial</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>tecido com proteção uv</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Comercial</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>roupa com proteção uv funciona</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Comercial</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>a proteção uv da roupa sai na lavagem</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Comercial</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>como funciona a roupa com proteção solar</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Comercial</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>roupa uv vale a pena</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Comercial</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>camiseta com proteção solar</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Comercial</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>legging com proteção uv</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Comercial</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>como se proteger do sol</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Comportamento</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>como se proteger do sol na praia</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Comportamento</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>como se proteger do sol no dia a dia</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Comportamento</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>melhor horário para tomar sol</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Comportamento</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>quanto tempo pode ficar no sol</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>Comportamento</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>proteção solar no inverno</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Comportamento</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>proteção solar em dia nublado</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Comportamento</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>como proteger o rosto do sol</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Comportamento</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>como proteger os olhos do sol</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>proteção solar</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>Comportamento</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (proposta de valor da marca)</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>melhor protetor solar</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>protetor solar</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Adjacente-creme</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (ponte: roupa complementa o creme)</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>protetor solar corporal</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>protetor solar</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>Adjacente-creme</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (ponte: roupa complementa o creme)</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>protetor solar facial</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>protetor solar</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Adjacente-creme</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (ponte: roupa complementa o creme)</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>como passar protetor solar</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>protetor solar</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>Adjacente-creme</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (ponte: roupa complementa o creme)</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>quando reaplicar protetor solar</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>protetor solar</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>Adjacente-creme</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (ponte: roupa complementa o creme)</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>protetor solar resistente à água</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>protetor solar</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>Adjacente-creme</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (ponte: roupa complementa o creme)</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>protetor solar fps 50</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>protetor solar</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Adjacente-creme</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (ponte: roupa complementa o creme)</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>protetor solar para pele oleosa</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>protetor solar</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Adjacente-creme</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (ponte: roupa complementa o creme)</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>protetor solar com cor</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>protetor solar</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Adjacente-creme</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (ponte: roupa complementa o creme)</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>protetor solar em spray</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>protetor solar</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Adjacente-creme</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (ponte: roupa complementa o creme)</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>protetor solar e roupa uv juntos</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>protetor solar</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Adjacente-creme</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (ponte: roupa complementa o creme)</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>protetor solar não é suficiente</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>protetor solar</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Adjacente-creme</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (ponte: roupa complementa o creme)</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>como prevenir câncer de pele</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>pele e saúde</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Saúde</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (autoridade em fotoproteção)</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>câncer de pele prevenção</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>pele e saúde</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>Saúde</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (autoridade em fotoproteção)</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>manchas de sol na pele</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>pele e saúde</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>Saúde</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (autoridade em fotoproteção)</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>melasma e sol</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>pele e saúde</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Saúde</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (autoridade em fotoproteção)</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>envelhecimento da pele pelo sol</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>pele e saúde</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>Saúde</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (autoridade em fotoproteção)</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>queimadura de sol o que fazer</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>pele e saúde</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Saúde</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (autoridade em fotoproteção)</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>como tratar queimadura de sol</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>pele e saúde</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Saúde</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (autoridade em fotoproteção)</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>pele sensível ao sol</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>pele e saúde</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Saúde</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (autoridade em fotoproteção)</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>alergia ao sol</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>pele e saúde</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Saúde</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (autoridade em fotoproteção)</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>insolação sintomas</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>pele e saúde</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Saúde</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>camiseta UV / lycra (autoridade em fotoproteção)</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>proteção solar para bebê</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>proteção infantil</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Família</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>camiseta UV infantil / maiô infantil</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>protetor solar infantil</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>proteção infantil</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>Família</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>camiseta UV infantil / maiô infantil</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>roupa com proteção uv infantil</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>proteção infantil</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>Família</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>camiseta UV infantil / maiô infantil</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>como proteger o bebê do sol</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>proteção infantil</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Família</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>camiseta UV infantil / maiô infantil</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>bebê pode tomar sol</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>proteção infantil</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Família</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>camiseta UV infantil / maiô infantil</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>criança pode usar protetor solar</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>proteção infantil</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Família</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>camiseta UV infantil / maiô infantil</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>primeira ida à praia do bebê</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>proteção infantil</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Família</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>camiseta UV infantil / maiô infantil</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>roupa de praia para bebê</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>proteção infantil</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Família</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>camiseta UV infantil / maiô infantil</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>proteção solar para crianças na escola</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>proteção infantil</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Família</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>camiseta UV infantil / maiô infantil</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>dicas para o verão</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>verão</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Estação</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>saída de praia / poncho / maiô / biquíni</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>cuidados no verão</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>verão</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Estação</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>saída de praia / poncho / maiô / biquíni</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>como se refrescar no calor</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>verão</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Estação</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>saída de praia / poncho / maiô / biquíni</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>hidratação no verão</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>verão</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Estação</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>saída de praia / poncho / maiô / biquíni</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>o que fazer no verão</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>verão</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Estação</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>saída de praia / poncho / maiô / biquíni</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>alimentação no verão</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>verão</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Estação</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>saída de praia / poncho / maiô / biquíni</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>cuidados com a pele no verão</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>verão</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>Estação</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>saída de praia / poncho / maiô / biquíni</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>cuidados com o cabelo no verão</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>verão</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>Estação</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>saída de praia / poncho / maiô / biquíni</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>cabelo no mar como cuidar</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>verão</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Estação</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>saída de praia / poncho / maiô / biquíni</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>cabelo na piscina cloro</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>verão</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>Estação</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>saída de praia / poncho / maiô / biquíni</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>pele oleosa no verão</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>verão</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>Estação</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>saída de praia / poncho / maiô / biquíni</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>maquiagem para o verão à prova d'água</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>verão</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>Estação</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>saída de praia / poncho / maiô / biquíni</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>o que levar para a praia</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>dia de praia</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>Estação</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>saída de praia / poncho / maiô / biquíni</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>checklist de praia</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>dia de praia</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Estação</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>saída de praia / poncho / maiô / biquíni</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>o que levar na bolsa de praia</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>dia de praia</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Estação</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>saída de praia / poncho / maiô / biquíni</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>dia de praia dicas</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>dia de praia</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Estação</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>saída de praia / poncho / maiô / biquíni</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>praia ou piscina</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>dia de praia</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Estação</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>saída de praia / poncho / maiô / biquíni</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>como montar um dia de praia perfeito</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>dia de praia</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>Estação</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>saída de praia / poncho / maiô / biquíni</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>o que levar para a praia com criança</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>dia de praia</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Estação</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>saída de praia / poncho / maiô / biquíni</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>dia de praia com cachorro</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>dia de praia</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>Estação</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>saída de praia / poncho / maiô / biquíni</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>o que vestir na praia</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>moda de verão</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Look</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>saída de praia / vestido / biquíni / maiô</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>look de praia</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>moda de verão</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Look</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>saída de praia / vestido / biquíni / maiô</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>tendências moda praia verão</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>moda de verão</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>Look</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>saída de praia / vestido / biquíni / maiô</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>como usar saída de praia</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>moda de verão</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Look</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>saída de praia / vestido / biquíni / maiô</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>o que usar na praia à noite</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>moda de verão</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>Look</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>saída de praia / vestido / biquíni / maiô</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>look praia dia</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>moda de verão</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Look</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>saída de praia / vestido / biquíni / maiô</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>cores tendência verão</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>moda de verão</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Look</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>saída de praia / vestido / biquíni / maiô</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>como escolher biquíni para o corpo</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>moda de verão</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Look</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>saída de praia / vestido / biquíni / maiô</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>o que vestir em dia de calor</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>moda de verão</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Look</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>saída de praia / vestido / biquíni / maiô</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
         <is>
           <t>não</t>
         </is>
@@ -9728,7 +12159,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A86"/>
+  <dimension ref="A1:A101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -10333,6 +12764,111 @@
       <c r="A86" t="inlineStr">
         <is>
           <t>atividades ao ar livre no verão</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>o que é fps</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>o que é fpu</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>o que é upf</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>diferença entre uva e uvb</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>o que é índice uv</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>o que é radiação ultravioleta</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>o que é fotoproteção</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>fps qual o ideal</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>fps 30 ou 50</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>o que é fator de proteção uv na roupa</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>roupa com fps</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>tecido com proteção uv</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>roupa com proteção uv funciona</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>a proteção uv da roupa sai na lavagem</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>como funciona a roupa com proteção solar</t>
         </is>
       </c>
     </row>
@@ -10347,7 +12883,528 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:A72"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>roupa uv vale a pena</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>camiseta com proteção solar</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>legging com proteção uv</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>como se proteger do sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>como se proteger do sol na praia</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>como se proteger do sol no dia a dia</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>melhor horário para tomar sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>quanto tempo pode ficar no sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>proteção solar no inverno</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>proteção solar em dia nublado</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>como proteger o rosto do sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>como proteger os olhos do sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>melhor protetor solar</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>protetor solar corporal</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>protetor solar facial</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>como passar protetor solar</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>quando reaplicar protetor solar</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>protetor solar resistente à água</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>protetor solar fps 50</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>protetor solar para pele oleosa</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>protetor solar com cor</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>protetor solar em spray</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>protetor solar e roupa uv juntos</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>protetor solar não é suficiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>como prevenir câncer de pele</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>câncer de pele prevenção</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>manchas de sol na pele</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>melasma e sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>envelhecimento da pele pelo sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>queimadura de sol o que fazer</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>como tratar queimadura de sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>pele sensível ao sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>alergia ao sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>insolação sintomas</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>proteção solar para bebê</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>protetor solar infantil</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>roupa com proteção uv infantil</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>como proteger o bebê do sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>bebê pode tomar sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>criança pode usar protetor solar</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>primeira ida à praia do bebê</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>roupa de praia para bebê</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>proteção solar para crianças na escola</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>dicas para o verão</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>cuidados no verão</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>como se refrescar no calor</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>hidratação no verão</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>o que fazer no verão</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>alimentação no verão</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>cuidados com a pele no verão</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>cuidados com o cabelo no verão</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>cabelo no mar como cuidar</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>cabelo na piscina cloro</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>pele oleosa no verão</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>maquiagem para o verão à prova d'água</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>o que levar para a praia</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>checklist de praia</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>o que levar na bolsa de praia</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>dia de praia dicas</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>praia ou piscina</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>como montar um dia de praia perfeito</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>o que levar para a praia com criança</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>dia de praia com cachorro</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>look de praia</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>tendências moda praia verão</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>como usar saída de praia</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>o que usar na praia à noite</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>look praia dia</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>cores tendência verão</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>como escolher biquíni para o corpo</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>o que vestir em dia de calor</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -10389,37 +13446,37 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>kitesurf</t>
+          <t>proteção solar</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>natação piscina</t>
+          <t>kitesurf</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>stand up paddle</t>
+          <t>natação piscina</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>futevôlei</t>
+          <t>stand up paddle</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -10429,27 +13486,27 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>pilates</t>
+          <t>futevôlei</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>canoa havaiana</t>
+          <t>pilates</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>treino funcional</t>
+          <t>canoa havaiana</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -10459,17 +13516,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>natação mar</t>
+          <t>treino funcional</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>canoagem</t>
+          <t>natação mar</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -10479,7 +13536,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>vôlei de praia</t>
+          <t>canoagem</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -10489,127 +13546,267 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>wakeboard</t>
+          <t>vôlei de praia</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>proteção solar esporte</t>
+          <t>wakeboard</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>verão e praia</t>
+          <t>protetor solar</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>verão</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>etapa</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>termos</t>
-        </is>
+          <t>pele e saúde</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Prática</t>
+          <t>proteção infantil</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>63</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Iniciante</t>
+          <t>moda de verão</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>49</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Equipamento</t>
+          <t>dia de praia</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Descoberta</t>
+          <t>proteção solar esporte</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>39</v>
+        <v>7</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Benefícios</t>
+          <t>verão e praia</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Adjacente</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>28</v>
-      </c>
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Local</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>22</v>
+          <t>etapa</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>termos</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>Prática</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Iniciante</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Equipamento</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Descoberta</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Benefícios</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Adjacente</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>Comportamento</t>
         </is>
       </c>
-      <c r="B26" t="n">
+      <c r="B33" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Estação</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Adjacente-creme</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
         <v>12</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Fundamento</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Comercial</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Saúde</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Família</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Look</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>